<commit_message>
Publish audited trend-p interval corrections through immutable overlays
</commit_message>
<xml_diff>
--- a/summary/no/exposures_meta_analysis_bladder_cancer_combined.xlsx
+++ b/summary/no/exposures_meta_analysis_bladder_cancer_combined.xlsx
@@ -452,84 +452,60 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Exposure</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>number estimates</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Pooled RR</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>lower CI RR</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>upper CI RR</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>lower PI RR</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>upper PI RR</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>I^2 (%)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>eggers p-value</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>total N</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>total Cases</t>
-        </is>
+      <c r="A1" s="1" t="str">
+        <v>Exposure</v>
+      </c>
+      <c r="B1" s="1" t="str">
+        <v>number estimates</v>
+      </c>
+      <c r="C1" s="1" t="str">
+        <v>Pooled RR</v>
+      </c>
+      <c r="D1" s="1" t="str">
+        <v>lower CI RR</v>
+      </c>
+      <c r="E1" s="1" t="str">
+        <v>upper CI RR</v>
+      </c>
+      <c r="F1" s="1" t="str">
+        <v>lower PI RR</v>
+      </c>
+      <c r="G1" s="1" t="str">
+        <v>upper PI RR</v>
+      </c>
+      <c r="H1" s="1" t="str">
+        <v>I^2 (%)</v>
+      </c>
+      <c r="I1" s="1" t="str">
+        <v>eggers p-value</v>
+      </c>
+      <c r="J1" s="1" t="str">
+        <v>total N</v>
+      </c>
+      <c r="K1" s="1" t="str">
+        <v>total Cases</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>zeaxanthin</t>
-        </is>
+      <c r="A2" t="str">
+        <v>zeaxanthin</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.1606125118752876</v>
+        <v>0.160612511875288</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.02008938167695712</v>
+        <v>0.020089381676957</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>1.059711334632446</v>
       </c>
-      <c r="F2" s="3" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" s="5" t="inlineStr"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="5"/>
       <c r="J2" s="2" t="n">
         <v>257</v>
       </c>
@@ -538,27 +514,25 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>alpha_linolenic_acid</t>
-        </is>
+      <c r="A3" t="str">
+        <v>alpha_linolenic_acid</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0.2608764404894685</v>
+        <v>0.260876440489468</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.1004102763893268</v>
+        <v>0.100410276389327</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.6510344938106651</v>
-      </c>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr"/>
+        <v>0.651034493810665</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="5"/>
       <c r="J3" s="2" t="n">
         <v>561</v>
       </c>
@@ -567,29 +541,27 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>omega_3_fatty_acids</t>
-        </is>
+      <c r="A4" t="str">
+        <v>omega_3_fatty_acids</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.3063889211181519</v>
+        <v>0.306388921118152</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.1968132439764496</v>
+        <v>0.19681324397645</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.4770185022795724</v>
-      </c>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
+        <v>0.477018502279572</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
       <c r="H4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="5" t="inlineStr"/>
+      <c r="I4" s="5"/>
       <c r="J4" s="2" t="n">
         <v>1061</v>
       </c>
@@ -598,27 +570,25 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>eicosapentaenoic_acid</t>
-        </is>
+      <c r="A5" t="str">
+        <v>eicosapentaenoic_acid</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>0.3209909633019056</v>
+        <v>0.320990963301906</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>0.19070128490511</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.5211356588277174</v>
-      </c>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr"/>
+        <v>0.521135658827717</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="5"/>
       <c r="J5" s="2" t="n">
         <v>500</v>
       </c>
@@ -627,10 +597,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>docosahexaenoic_acid</t>
-        </is>
+      <c r="A6" t="str">
+        <v>docosahexaenoic_acid</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>1</v>
@@ -642,12 +610,12 @@
         <v>0.20072904790198</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.5311333323044712</v>
-      </c>
-      <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr"/>
+        <v>0.531133332304471</v>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="5"/>
       <c r="J6" s="2" t="n">
         <v>500</v>
       </c>
@@ -656,27 +624,25 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>multivitamin</t>
-        </is>
+      <c r="A7" t="str">
+        <v>multivitamin</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.3910830654414335</v>
+        <v>0.391083065441434</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>0.2408309631552709</v>
+        <v>0.240830963155271</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.6310600546798513</v>
-      </c>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr"/>
+        <v>0.631060054679851</v>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="5"/>
       <c r="J7" s="2" t="n">
         <v>667</v>
       </c>
@@ -685,27 +651,25 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>linoleic_acid</t>
-        </is>
+      <c r="A8" t="str">
+        <v>linoleic_acid</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.4311156410559245</v>
+        <v>0.431115641055925</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>0.19070128490511</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.9601743676651679</v>
-      </c>
-      <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr"/>
+        <v>0.960174367665168</v>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="5"/>
       <c r="J8" s="2" t="n">
         <v>561</v>
       </c>
@@ -714,27 +678,25 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>dihomo_gamma_linolenic_acid</t>
-        </is>
+      <c r="A9" t="str">
+        <v>dihomo_gamma_linolenic_acid</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.4711336417688241</v>
+        <v>0.471133641768824</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.2909378089333156</v>
+        <v>0.290937808933316</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.7408745282931972</v>
-      </c>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" s="5" t="inlineStr"/>
+        <v>0.740874528293197</v>
+      </c>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="5"/>
       <c r="J9" s="2" t="n">
         <v>500</v>
       </c>
@@ -743,27 +705,25 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>olive</t>
-        </is>
+      <c r="A10" t="str">
+        <v>olive</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.4711336417688241</v>
+        <v>0.471133641768824</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.2809182656266805</v>
+        <v>0.28091826562668</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.7807798429070956</v>
-      </c>
-      <c r="F10" s="3" t="inlineStr"/>
-      <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="5" t="inlineStr"/>
+        <v>0.780779842907096</v>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="5"/>
       <c r="J10" s="2" t="n">
         <v>586</v>
       </c>
@@ -772,27 +732,25 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>olive_oil_intake</t>
-        </is>
+      <c r="A11" t="str">
+        <v>olive_oil_intake</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.4711336417688241</v>
+        <v>0.471133641768824</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.2809182656266805</v>
+        <v>0.28091826562668</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.7807798429070956</v>
-      </c>
-      <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="4" t="inlineStr"/>
-      <c r="I11" s="5" t="inlineStr"/>
+        <v>0.780779842907096</v>
+      </c>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="5"/>
       <c r="J11" s="2" t="n">
         <v>586</v>
       </c>
@@ -801,10 +759,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>oleic_acid</t>
-        </is>
+      <c r="A12" t="str">
+        <v>oleic_acid</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>1</v>
@@ -813,15 +769,15 @@
         <v>0.54113009609268</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.3410218378348885</v>
+        <v>0.341021837834888</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>0.860546963650096</v>
       </c>
-      <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="5" t="inlineStr"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="5"/>
       <c r="J12" s="2" t="n">
         <v>500</v>
       </c>
@@ -830,27 +786,25 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>vitamin_b3</t>
-        </is>
+      <c r="A13" t="str">
+        <v>vitamin_b3</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.5611208951000519</v>
+        <v>0.561120895100052</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.3109741576462426</v>
+        <v>0.310974157646243</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>1.019907392408769</v>
       </c>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" s="5" t="inlineStr"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="5"/>
       <c r="J13" s="2" t="n">
         <v>561</v>
       </c>
@@ -859,29 +813,27 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>legumes</t>
-        </is>
+      <c r="A14" t="str">
+        <v>legumes</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.6397997770084459</v>
+        <v>0.639799777008446</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0.4305034246903502</v>
+        <v>0.43050342469035</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.9507539286723269</v>
-      </c>
-      <c r="F14" s="3" t="inlineStr"/>
-      <c r="G14" s="3" t="inlineStr"/>
+        <v>0.950753928672327</v>
+      </c>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
       <c r="H14" s="4" t="n">
         <v>77.91</v>
       </c>
-      <c r="I14" s="5" t="inlineStr"/>
+      <c r="I14" s="5"/>
       <c r="J14" s="2" t="n">
         <v>2541</v>
       </c>
@@ -890,29 +842,27 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>yogurt</t>
-        </is>
+      <c r="A15" t="str">
+        <v>yogurt</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0.6435857533404954</v>
+        <v>0.643585753340495</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0.2494242542659014</v>
+        <v>0.249424254265901</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>1.660634901453039</v>
       </c>
-      <c r="F15" s="3" t="inlineStr"/>
-      <c r="G15" s="3" t="inlineStr"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
       <c r="H15" s="4" t="n">
         <v>70.34</v>
       </c>
-      <c r="I15" s="5" t="inlineStr"/>
+      <c r="I15" s="5"/>
       <c r="J15" s="2" t="n">
         <v>101981</v>
       </c>
@@ -921,34 +871,32 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>lutein</t>
-        </is>
+      <c r="A16" t="str">
+        <v>lutein</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.6941272346837586</v>
+        <v>0.694127234683759</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.3791588622931857</v>
+        <v>0.379158862293186</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>1.270740752347649</v>
+        <v>1.27074075234765</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.0007090691841002699</v>
+        <v>0.000709069184001</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>679.5001513725188</v>
+        <v>679.5001514673125</v>
       </c>
       <c r="H16" s="4" t="n">
         <v>71.59</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.1894295826083661</v>
+        <v>0.189429582608366</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>122821</v>
@@ -958,28 +906,26 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>vitamin_a</t>
-        </is>
+      <c r="A17" t="str">
+        <v>vitamin_a</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>4</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>0.7164835434120075</v>
+        <v>0.716483543412008</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>0.5214718421284985</v>
+        <v>0.521471842128498</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.9843241652031548</v>
+        <v>0.984324165203155</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>0.2212620745858667</v>
+        <v>0.221262074589089</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>2.320093350571054</v>
+        <v>2.320093350537271</v>
       </c>
       <c r="H17" s="4" t="n">
         <v>46.43</v>
@@ -995,34 +941,32 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>whole_grain_intake</t>
-        </is>
+      <c r="A18" t="str">
+        <v>whole_grain_intake</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0.7226718735643111</v>
+        <v>0.722671873564311</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0.5177307290339085</v>
+        <v>0.517730729033908</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>1.008737954989623</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>0.01658634469437209</v>
+        <v>0.016586344693104</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>31.48702420360033</v>
+        <v>31.487024206007852</v>
       </c>
       <c r="H18" s="4" t="n">
         <v>75.47</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.2822678427106021</v>
+        <v>0.282267842710602</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>219042</v>
@@ -1032,10 +976,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>selenium</t>
-        </is>
+      <c r="A19" t="str">
+        <v>selenium</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>8</v>
@@ -1044,22 +986,22 @@
         <v>0.725713478332136</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0.5422110294998878</v>
+        <v>0.542211029499888</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.9713193276770786</v>
+        <v>0.971319327677079</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>0.2945606787230922</v>
+        <v>0.294560678723093</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>1.787950974705708</v>
+        <v>1.787950974705702</v>
       </c>
       <c r="H19" s="4" t="n">
         <v>71.62</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>0.1356590524221063</v>
+        <v>0.135659052422106</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>161440</v>
@@ -1069,34 +1011,32 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>dairy</t>
-        </is>
+      <c r="A20" t="str">
+        <v>dairy</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>8</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0.7336670233195703</v>
+        <v>0.73366702331957</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0.5325385444896668</v>
+        <v>0.532538544489667</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>1.010757449721169</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>0.2667027912984513</v>
+        <v>0.266702791298452</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>2.018228974980078</v>
+        <v>2.01822897498007</v>
       </c>
       <c r="H20" s="4" t="n">
         <v>80.88</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.03414991977459563</v>
+        <v>0.034149919774596</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>306953</v>
@@ -1106,34 +1046,32 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>fermented_foods</t>
-        </is>
+      <c r="A21" t="str">
+        <v>fermented_foods</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>0.7490122054026693</v>
+        <v>0.749012205402669</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.5024294735717695</v>
+        <v>0.50242947357177</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>1.116613004117546</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>0.1999700203677981</v>
+        <v>0.199970020367752</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>2.805516961043995</v>
+        <v>2.805516961044641</v>
       </c>
       <c r="H21" s="4" t="n">
         <v>73.37</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>0.6646008321307554</v>
+        <v>0.664600832130755</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>203999</v>
@@ -1143,27 +1081,25 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>non_nutritive_sweetener_intake</t>
-        </is>
+      <c r="A22" t="str">
+        <v>non_nutritive_sweetener_intake</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>0.7504264322028401</v>
+        <v>0.75042643220284</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>0.5305667184532947</v>
+        <v>0.530566718453295</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>1.059855422172594</v>
       </c>
-      <c r="F22" s="3" t="inlineStr"/>
-      <c r="G22" s="3" t="inlineStr"/>
-      <c r="H22" s="4" t="inlineStr"/>
-      <c r="I22" s="5" t="inlineStr"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="5"/>
       <c r="J22" s="2" t="n">
         <v>80388</v>
       </c>
@@ -1172,34 +1108,32 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>vitamin_c</t>
-        </is>
+      <c r="A23" t="str">
+        <v>vitamin_c</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>0.7509621709935039</v>
+        <v>0.750962170993504</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0.5556037048097945</v>
+        <v>0.555603704809794</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>1.014910062303704</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>0.05110412975560341</v>
+        <v>0.051104129752821</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>11.03519783939657</v>
+        <v>11.035197839997357</v>
       </c>
       <c r="H23" s="4" t="n">
         <v>26.75</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>0.7498815991687291</v>
+        <v>0.749881599168729</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>8606</v>
@@ -1209,34 +1143,32 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>vitamin_d</t>
-        </is>
+      <c r="A24" t="str">
+        <v>vitamin_d</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>10</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>0.7519390566538966</v>
+        <v>0.751939056653897</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>0.3459019242605473</v>
+        <v>0.345901924260547</v>
       </c>
       <c r="E24" s="3" t="n">
         <v>1.634439610946421</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>0.03851548454774519</v>
+        <v>0.038515484547745</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>14.68013064253797</v>
+        <v>14.680130642537975</v>
       </c>
       <c r="H24" s="4" t="n">
         <v>98.12</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.01068136703040478</v>
+        <v>0.010681367030405</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>339695</v>
@@ -1246,34 +1178,32 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>vitamin_e</t>
-        </is>
+      <c r="A25" t="str">
+        <v>vitamin_e</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>5</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>0.7637612795223642</v>
+        <v>0.763761279522364</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0.5830980062410815</v>
+        <v>0.583098006241082</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>1.0003000450045</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>0.350245514116067</v>
+        <v>0.350245514116019</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>1.665492543337272</v>
+        <v>1.665492543337498</v>
       </c>
       <c r="H25" s="4" t="n">
         <v>43.82</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>0.6652833451872155</v>
+        <v>0.665283345187216</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>158299</v>
@@ -1283,27 +1213,25 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>vitamin_b12</t>
-        </is>
+      <c r="A26" t="str">
+        <v>vitamin_b12</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>0.7708048744499005</v>
+        <v>0.7708048744499</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.6110819817568988</v>
+        <v>0.611081981756899</v>
       </c>
       <c r="E26" s="3" t="n">
         <v>0.990044948040641</v>
       </c>
-      <c r="F26" s="3" t="inlineStr"/>
-      <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="5" t="inlineStr"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="5"/>
       <c r="J26" s="2" t="n">
         <v>2589</v>
       </c>
@@ -1312,34 +1240,32 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>folic_acid</t>
-        </is>
+      <c r="A27" t="str">
+        <v>folic_acid</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>5</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>0.7732908808107848</v>
+        <v>0.773290880810785</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>0.6068340008714599</v>
+        <v>0.60683400087146</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.9854075175194142</v>
+        <v>0.985407517519414</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>0.3516080413086398</v>
+        <v>0.351608041308591</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>1.700697128881124</v>
+        <v>1.700697128881358</v>
       </c>
       <c r="H27" s="4" t="n">
         <v>63.72</v>
       </c>
       <c r="I27" s="5" t="n">
-        <v>0.2913323489409054</v>
+        <v>0.291332348940905</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>309245</v>
@@ -1349,29 +1275,27 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>avocado</t>
-        </is>
+      <c r="A28" t="str">
+        <v>avocado</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>0.7773224664291063</v>
+        <v>0.777322466429106</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0.5959491108750986</v>
+        <v>0.595949110875099</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>1.013794275030678</v>
       </c>
-      <c r="F28" s="3" t="inlineStr"/>
-      <c r="G28" s="3" t="inlineStr"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
       <c r="H28" s="4" t="n">
         <v>20.99</v>
       </c>
-      <c r="I28" s="5" t="inlineStr"/>
+      <c r="I28" s="5"/>
       <c r="J28" s="2" t="n">
         <v>112328</v>
       </c>
@@ -1380,27 +1304,25 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>insoluble_dietary_fiber_intake</t>
-        </is>
+      <c r="A29" t="str">
+        <v>insoluble_dietary_fiber_intake</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>0.8303208655186842</v>
+        <v>0.830320865518684</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0.6705029098644103</v>
+        <v>0.67050290986441</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>1.029929753803904</v>
       </c>
-      <c r="F29" s="3" t="inlineStr"/>
-      <c r="G29" s="3" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr"/>
-      <c r="I29" s="5" t="inlineStr"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="5"/>
       <c r="J29" s="2" t="n">
         <v>101721</v>
       </c>
@@ -1409,34 +1331,32 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>beta_carotene</t>
-        </is>
+      <c r="A30" t="str">
+        <v>beta_carotene</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>6</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>0.8304396663075081</v>
+        <v>0.830439666307508</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>0.6609348544756805</v>
+        <v>0.66093485447568</v>
       </c>
       <c r="E30" s="3" t="n">
         <v>1.04352040319657</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>0.4275552528813619</v>
+        <v>0.427555252881361</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>1.612961213151751</v>
+        <v>1.612961213151754</v>
       </c>
       <c r="H30" s="4" t="n">
         <v>58.87</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.8823731624979889</v>
+        <v>0.882373162497989</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>368253</v>
@@ -1446,29 +1366,27 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>plant_protein_intake</t>
-        </is>
+      <c r="A31" t="str">
+        <v>plant_protein_intake</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>0.8387018493286374</v>
+        <v>0.838701849328638</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0.7048290414313586</v>
+        <v>0.704829041431359</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0.9981018038573761</v>
-      </c>
-      <c r="F31" s="3" t="inlineStr"/>
-      <c r="G31" s="3" t="inlineStr"/>
+        <v>0.998101803857376</v>
+      </c>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
       <c r="H31" s="4" t="n">
         <v>38.28</v>
       </c>
-      <c r="I31" s="5" t="inlineStr"/>
+      <c r="I31" s="5"/>
       <c r="J31" s="2" t="n">
         <v>585408</v>
       </c>
@@ -1477,29 +1395,27 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>total_dietary_fiber_intake</t>
-        </is>
+      <c r="A32" t="str">
+        <v>total_dietary_fiber_intake</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>0.8530816628701524</v>
+        <v>0.853081662870152</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>0.7636085425406669</v>
+        <v>0.763608542540667</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0.9529431793814942</v>
-      </c>
-      <c r="F32" s="3" t="inlineStr"/>
-      <c r="G32" s="3" t="inlineStr"/>
+        <v>0.952943179381494</v>
+      </c>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
       <c r="H32" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I32" s="5" t="inlineStr"/>
+      <c r="I32" s="5"/>
       <c r="J32" s="2" t="n">
         <v>676447</v>
       </c>
@@ -1508,93 +1424,87 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>soluble_dietary_fiber_intake</t>
-        </is>
+      <c r="A33" t="str">
+        <v>alcohol</v>
       </c>
       <c r="B33" s="2" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C33" s="3" t="n">
+        <v>0.858644754138728</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>0.739929771992727</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>0.996306836565637</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>0.526355059174737</v>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>1.400710035856616</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>0.101649926298899</v>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>882294</v>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>8649</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>soluble_dietary_fiber_intake</v>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="3" t="n">
         <v>0.86027378065949</v>
       </c>
-      <c r="D33" s="3" t="n">
-        <v>0.6804949413246006</v>
-      </c>
-      <c r="E33" s="3" t="n">
+      <c r="D34" s="3" t="n">
+        <v>0.680494941324601</v>
+      </c>
+      <c r="E34" s="3" t="n">
         <v>1.079803598340883</v>
       </c>
-      <c r="F33" s="3" t="inlineStr"/>
-      <c r="G33" s="3" t="inlineStr"/>
-      <c r="H33" s="4" t="inlineStr"/>
-      <c r="I33" s="5" t="inlineStr"/>
-      <c r="J33" s="2" t="n">
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="2" t="n">
         <v>101721</v>
       </c>
-      <c r="K33" s="2" t="n">
+      <c r="K34" s="2" t="n">
         <v>776</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>alcohol</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="C34" s="3" t="n">
-        <v>0.8798533791446438</v>
-      </c>
-      <c r="D34" s="3" t="n">
-        <v>0.760104009849826</v>
-      </c>
-      <c r="E34" s="3" t="n">
-        <v>1.018366629349689</v>
-      </c>
-      <c r="F34" s="3" t="n">
-        <v>0.5430280916493282</v>
-      </c>
-      <c r="G34" s="3" t="n">
-        <v>1.425602064970456</v>
-      </c>
-      <c r="H34" s="4" t="n">
-        <v>83.81</v>
-      </c>
-      <c r="I34" s="5" t="n">
-        <v>0.1667217348872468</v>
-      </c>
-      <c r="J34" s="2" t="n">
-        <v>1003146</v>
-      </c>
-      <c r="K34" s="2" t="n">
-        <v>9243</v>
-      </c>
-    </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>mediterranean_diet</t>
-        </is>
+      <c r="A35" t="str">
+        <v>mediterranean_diet</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>0.8902226072035401</v>
+        <v>0.89022260720354</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>0.6205359319277568</v>
+        <v>0.620535931927757</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>1.259255513560131</v>
       </c>
-      <c r="F35" s="3" t="inlineStr"/>
-      <c r="G35" s="3" t="inlineStr"/>
-      <c r="H35" s="4" t="inlineStr"/>
-      <c r="I35" s="5" t="inlineStr"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="4"/>
+      <c r="I35" s="5"/>
       <c r="J35" s="2" t="n">
         <v>37442</v>
       </c>
@@ -1603,16 +1513,14 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>monounsaturated_fat_mufa</t>
-        </is>
+      <c r="A36" t="str">
+        <v>monounsaturated_fat_mufa</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>0.9462958698523343</v>
+        <v>0.946295869852334</v>
       </c>
       <c r="D36" s="3" t="n">
         <v>0.436660182850176</v>
@@ -1620,12 +1528,12 @@
       <c r="E36" s="3" t="n">
         <v>2.050943641160259</v>
       </c>
-      <c r="F36" s="3" t="inlineStr"/>
-      <c r="G36" s="3" t="inlineStr"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
       <c r="H36" s="4" t="n">
         <v>88.7</v>
       </c>
-      <c r="I36" s="5" t="inlineStr"/>
+      <c r="I36" s="5"/>
       <c r="J36" s="2" t="n">
         <v>648914</v>
       </c>
@@ -1634,34 +1542,32 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>lycopene</t>
-        </is>
+      <c r="A37" t="str">
+        <v>lycopene</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>0.9475268544497669</v>
+        <v>0.947526854449767</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0.9003245225862656</v>
+        <v>0.900324522586266</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0.9973036417217132</v>
+        <v>0.997303641721713</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>0.6800887710883596</v>
+        <v>0.680088771083791</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>1.320132279888537</v>
+        <v>1.320132279897406</v>
       </c>
       <c r="H37" s="4" t="n">
         <v>0</v>
       </c>
       <c r="I37" s="5" t="n">
-        <v>0.03008236612500683</v>
+        <v>0.030082366125007</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>222792</v>
@@ -1671,25 +1577,23 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>tea</t>
-        </is>
+      <c r="A38" t="str">
+        <v>tea</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>9</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>0.9617507091463667</v>
+        <v>0.961750709146367</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>0.7890701910914995</v>
+        <v>0.7890701910915</v>
       </c>
       <c r="E38" s="3" t="n">
         <v>1.172337946680718</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>0.5117552101281551</v>
+        <v>0.511755210128155</v>
       </c>
       <c r="G38" s="3" t="n">
         <v>1.807435289836927</v>
@@ -1698,7 +1602,7 @@
         <v>83.53</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.02398376617759525</v>
+        <v>0.023983766177595</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>580076</v>
@@ -1708,29 +1612,27 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>phosphorus</t>
-        </is>
+      <c r="A39" t="str">
+        <v>phosphorus</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>0.9740428329225616</v>
+        <v>0.974042832922562</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>0.2712267749764213</v>
+        <v>0.271226774976421</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>3.498030164795818</v>
       </c>
-      <c r="F39" s="3" t="inlineStr"/>
-      <c r="G39" s="3" t="inlineStr"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
       <c r="H39" s="4" t="n">
-        <v>82.45999999999999</v>
-      </c>
-      <c r="I39" s="5" t="inlineStr"/>
+        <v>82.46</v>
+      </c>
+      <c r="I39" s="5"/>
       <c r="J39" s="2" t="n">
         <v>1147</v>
       </c>
@@ -1739,10 +1641,8 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>magnesium</t>
-        </is>
+      <c r="A40" t="str">
+        <v>magnesium</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>1</v>
@@ -1756,10 +1656,10 @@
       <c r="E40" s="3" t="n">
         <v>1.823130081227917</v>
       </c>
-      <c r="F40" s="3" t="inlineStr"/>
-      <c r="G40" s="3" t="inlineStr"/>
-      <c r="H40" s="4" t="inlineStr"/>
-      <c r="I40" s="5" t="inlineStr"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="5"/>
       <c r="J40" s="2" t="n">
         <v>574</v>
       </c>
@@ -1768,10 +1668,8 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>vitamin_b1</t>
-        </is>
+      <c r="A41" t="str">
+        <v>vitamin_b1</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>3</v>
@@ -1780,22 +1678,22 @@
         <v>1.026135700809198</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>0.8760781322122511</v>
+        <v>0.876078132212251</v>
       </c>
       <c r="E41" s="3" t="n">
         <v>1.201895627523871</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>0.1861215877235062</v>
+        <v>0.186121587717069</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5.657347378958563</v>
+        <v>5.657347379154214</v>
       </c>
       <c r="H41" s="4" t="n">
         <v>71.67</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.6179812083215527</v>
+        <v>0.617981208321553</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>575001</v>
@@ -1805,10 +1703,8 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>iron</t>
-        </is>
+      <c r="A42" t="str">
+        <v>iron</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>1</v>
@@ -1817,15 +1713,15 @@
         <v>1.049880653285851</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>0.9900225074278087</v>
+        <v>0.990022507427809</v>
       </c>
       <c r="E42" s="3" t="n">
         <v>1.119694504834913</v>
       </c>
-      <c r="F42" s="3" t="inlineStr"/>
-      <c r="G42" s="3" t="inlineStr"/>
-      <c r="H42" s="4" t="inlineStr"/>
-      <c r="I42" s="5" t="inlineStr"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="5"/>
       <c r="J42" s="2" t="n">
         <v>481419</v>
       </c>
@@ -1834,10 +1730,8 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>processed_meat_intake</t>
-        </is>
+      <c r="A43" t="str">
+        <v>processed_meat_intake</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>7</v>
@@ -1846,13 +1740,13 @@
         <v>1.086433159799911</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>0.9792189645694596</v>
+        <v>0.97921896456946</v>
       </c>
       <c r="E43" s="3" t="n">
         <v>1.205265651112213</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>0.8385628597437634</v>
+        <v>0.838562859743763</v>
       </c>
       <c r="G43" s="3" t="n">
         <v>1.407571295339136</v>
@@ -1861,7 +1755,7 @@
         <v>41.47</v>
       </c>
       <c r="I43" s="5" t="n">
-        <v>0.08383782424174292</v>
+        <v>0.083837824241743</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>938913</v>
@@ -1871,10 +1765,8 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>western_pattern_diet</t>
-        </is>
+      <c r="A44" t="str">
+        <v>western_pattern_diet</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>1</v>
@@ -1888,10 +1780,10 @@
       <c r="E44" s="3" t="n">
         <v>1.378808493040073</v>
       </c>
-      <c r="F44" s="3" t="inlineStr"/>
-      <c r="G44" s="3" t="inlineStr"/>
-      <c r="H44" s="4" t="inlineStr"/>
-      <c r="I44" s="5" t="inlineStr"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="4"/>
+      <c r="I44" s="5"/>
       <c r="J44" s="2" t="n">
         <v>388077</v>
       </c>
@@ -1900,10 +1792,8 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>sugar_sweetened_beverage_intake</t>
-        </is>
+      <c r="A45" t="str">
+        <v>sugar_sweetened_beverage_intake</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>1</v>
@@ -1917,10 +1807,10 @@
       <c r="E45" s="3" t="n">
         <v>1.219390011363415</v>
       </c>
-      <c r="F45" s="3" t="inlineStr"/>
-      <c r="G45" s="3" t="inlineStr"/>
-      <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="5" t="inlineStr"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="4"/>
+      <c r="I45" s="5"/>
       <c r="J45" s="2" t="n">
         <v>73024</v>
       </c>
@@ -1929,10 +1819,8 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>dietary_protein_intake</t>
-        </is>
+      <c r="A46" t="str">
+        <v>dietary_protein_intake</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>2</v>
@@ -1946,12 +1834,12 @@
       <c r="E46" s="3" t="n">
         <v>1.233678059956743</v>
       </c>
-      <c r="F46" s="3" t="inlineStr"/>
-      <c r="G46" s="3" t="inlineStr"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
       <c r="H46" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I46" s="5" t="inlineStr"/>
+      <c r="I46" s="5"/>
       <c r="J46" s="2" t="n">
         <v>585408</v>
       </c>
@@ -1960,10 +1848,8 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>animal_protein_intake</t>
-        </is>
+      <c r="A47" t="str">
+        <v>animal_protein_intake</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>2</v>
@@ -1977,12 +1863,12 @@
       <c r="E47" s="3" t="n">
         <v>1.277365814492968</v>
       </c>
-      <c r="F47" s="3" t="inlineStr"/>
-      <c r="G47" s="3" t="inlineStr"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
       <c r="H47" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I47" s="5" t="inlineStr"/>
+      <c r="I47" s="5"/>
       <c r="J47" s="2" t="n">
         <v>585408</v>
       </c>
@@ -1991,10 +1877,8 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>tomato</t>
-        </is>
+      <c r="A48" t="str">
+        <v>tomato</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>1</v>
@@ -2003,15 +1887,15 @@
         <v>1.19945453907786</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>0.9501079967336835</v>
+        <v>0.950107996733684</v>
       </c>
       <c r="E48" s="3" t="n">
         <v>1.518204486493061</v>
       </c>
-      <c r="F48" s="3" t="inlineStr"/>
-      <c r="G48" s="3" t="inlineStr"/>
-      <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" s="5" t="inlineStr"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="5"/>
       <c r="J48" s="2" t="n">
         <v>101683</v>
       </c>
@@ -2020,10 +1904,8 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>red_meat</t>
-        </is>
+      <c r="A49" t="str">
+        <v>red_meat</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>9</v>
@@ -2038,16 +1920,16 @@
         <v>1.570980583701342</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>0.7815874035063086</v>
+        <v>0.781587403506308</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>2.234524144537296</v>
+        <v>2.234524144537297</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>77.01000000000001</v>
+        <v>77.01</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>0.01127626650555045</v>
+        <v>0.01127626650555</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>1417360</v>
@@ -2057,188 +1939,172 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>soy</t>
-        </is>
+      <c r="A50" t="str">
+        <v>calcium</v>
       </c>
       <c r="B50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" s="3" t="n">
+        <v>1.763833989140762</v>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>3.119550071749652</v>
+      </c>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="5"/>
+      <c r="J50" s="2" t="n">
+        <v>586</v>
+      </c>
+      <c r="K50" s="2" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>caffeine</v>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>2.045114195119933</v>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>1.149607920243644</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>3.637955664073244</v>
+      </c>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="4"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="2" t="n">
+        <v>104440</v>
+      </c>
+      <c r="K51" s="2" t="n">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>pickled_vegetables</v>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>3.217136946095633</v>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>1.357780842990217</v>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>7.482070687809</v>
+      </c>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="4"/>
+      <c r="I52" s="5"/>
+      <c r="J52" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="K52" s="2" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>vegetable_and_seed_oil_intake</v>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>3.431519625226634</v>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>1.684722438489189</v>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>6.946365883186642</v>
+      </c>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="4"/>
+      <c r="I53" s="5"/>
+      <c r="J53" s="2" t="n">
+        <v>405</v>
+      </c>
+      <c r="K53" s="2" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>eggs</v>
+      </c>
+      <c r="B54" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C50" s="3" t="n">
-        <v>1.508325356558058</v>
-      </c>
-      <c r="D50" s="3" t="n">
-        <v>0.1884919459617998</v>
-      </c>
-      <c r="E50" s="3" t="n">
-        <v>12.0697219694313</v>
-      </c>
-      <c r="F50" s="3" t="inlineStr"/>
-      <c r="G50" s="3" t="inlineStr"/>
-      <c r="H50" s="4" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="I50" s="5" t="inlineStr"/>
-      <c r="J50" s="2" t="n">
-        <v>32477</v>
-      </c>
-      <c r="K50" s="2" t="n">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>calcium</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C51" s="3" t="n">
-        <v>1.763833989140762</v>
-      </c>
-      <c r="D51" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E51" s="3" t="n">
-        <v>3.119550071749652</v>
-      </c>
-      <c r="F51" s="3" t="inlineStr"/>
-      <c r="G51" s="3" t="inlineStr"/>
-      <c r="H51" s="4" t="inlineStr"/>
-      <c r="I51" s="5" t="inlineStr"/>
-      <c r="J51" s="2" t="n">
-        <v>586</v>
-      </c>
-      <c r="K51" s="2" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>caffeine</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C52" s="3" t="n">
-        <v>2.045114195119933</v>
-      </c>
-      <c r="D52" s="3" t="n">
-        <v>1.149607920243644</v>
-      </c>
-      <c r="E52" s="3" t="n">
-        <v>3.637955664073244</v>
-      </c>
-      <c r="F52" s="3" t="inlineStr"/>
-      <c r="G52" s="3" t="inlineStr"/>
-      <c r="H52" s="4" t="inlineStr"/>
-      <c r="I52" s="5" t="inlineStr"/>
-      <c r="J52" s="2" t="n">
-        <v>104440</v>
-      </c>
-      <c r="K52" s="2" t="n">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>pickled_vegetables</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C53" s="3" t="n">
-        <v>3.217136946095633</v>
-      </c>
-      <c r="D53" s="3" t="n">
-        <v>1.357780842990217</v>
-      </c>
-      <c r="E53" s="3" t="n">
-        <v>7.482070687809</v>
-      </c>
-      <c r="F53" s="3" t="inlineStr"/>
-      <c r="G53" s="3" t="inlineStr"/>
-      <c r="H53" s="4" t="inlineStr"/>
-      <c r="I53" s="5" t="inlineStr"/>
-      <c r="J53" s="2" t="n">
-        <v>260</v>
-      </c>
-      <c r="K53" s="2" t="n">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>vegetable_and_seed_oil_intake</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="C54" s="3" t="n">
-        <v>3.431519625226634</v>
+        <v>3.857811292537815</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>1.684722438489189</v>
+        <v>2.646928735129925</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>6.946365883186642</v>
-      </c>
-      <c r="F54" s="3" t="inlineStr"/>
-      <c r="G54" s="3" t="inlineStr"/>
-      <c r="H54" s="4" t="inlineStr"/>
-      <c r="I54" s="5" t="inlineStr"/>
+        <v>5.622632665288498</v>
+      </c>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="5"/>
       <c r="J54" s="2" t="n">
-        <v>405</v>
+        <v>1995</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>113</v>
+        <v>355</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>eggs</t>
-        </is>
+      <c r="A55" t="str">
+        <v>soy</v>
       </c>
       <c r="B55" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" s="3" t="n">
-        <v>3.857811292537815</v>
+        <v>4.61</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>2.646928735129925</v>
+        <v>1.57</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>5.622632665288498</v>
-      </c>
-      <c r="F55" s="3" t="inlineStr"/>
-      <c r="G55" s="3" t="inlineStr"/>
-      <c r="H55" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I55" s="5" t="inlineStr"/>
+        <v>13.51</v>
+      </c>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="4"/>
+      <c r="I55" s="5"/>
       <c r="J55" s="2" t="n">
-        <v>1995</v>
+        <v>18244</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>355</v>
+        <v>61</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>anti_inflammatory_diet</t>
-        </is>
+      <c r="A56" t="str">
+        <v>anti_inflammatory_diet</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>1</v>
@@ -2250,12 +2116,12 @@
         <v>1.456957290394739</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>20.44949521459941</v>
-      </c>
-      <c r="F56" s="3" t="inlineStr"/>
-      <c r="G56" s="3" t="inlineStr"/>
-      <c r="H56" s="4" t="inlineStr"/>
-      <c r="I56" s="5" t="inlineStr"/>
+        <v>20.449495214599413</v>
+      </c>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="H56" s="4"/>
+      <c r="I56" s="5"/>
       <c r="J56" s="2" t="n">
         <v>199</v>
       </c>

</xml_diff>

<commit_message>
Publish reviewed multisite evidence through conserved source overlays
</commit_message>
<xml_diff>
--- a/summary/no/exposures_meta_analysis_bladder_cancer_combined.xlsx
+++ b/summary/no/exposures_meta_analysis_bladder_cancer_combined.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Analysis mode" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$K$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$K$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -450,7 +450,7 @@
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
-  <sheetData>
+  <sheetData xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="str">
         <v>Exposure</v>
@@ -1012,295 +1012,295 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>dairy</v>
+        <v>fermented_foods</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0.73366702331957</v>
+        <v>0.749012205402669</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0.532538544489667</v>
+        <v>0.50242947357177</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>1.010757449721169</v>
+        <v>1.116613004117546</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>0.266702791298452</v>
+        <v>0.199970020367752</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>2.01822897498007</v>
+        <v>2.805516961044641</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>80.88</v>
+        <v>73.37</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.034149919774596</v>
+        <v>0.664600832130755</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>306953</v>
+        <v>203999</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>3788</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>fermented_foods</v>
+        <v>non_nutritive_sweetener_intake</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>0.749012205402669</v>
+        <v>0.75042643220284</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.50242947357177</v>
+        <v>0.530566718453295</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>1.116613004117546</v>
-      </c>
-      <c r="F21" s="3" t="n">
-        <v>0.199970020367752</v>
-      </c>
-      <c r="G21" s="3" t="n">
-        <v>2.805516961044641</v>
-      </c>
-      <c r="H21" s="4" t="n">
-        <v>73.37</v>
-      </c>
-      <c r="I21" s="5" t="n">
-        <v>0.664600832130755</v>
-      </c>
+        <v>1.059855422172594</v>
+      </c>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="5"/>
       <c r="J21" s="2" t="n">
-        <v>203999</v>
+        <v>80388</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>2474</v>
+        <v>448</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>non_nutritive_sweetener_intake</v>
+        <v>vitamin_c</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>0.75042643220284</v>
+        <v>0.750962170993504</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>0.530566718453295</v>
+        <v>0.555603704809794</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>1.059855422172594</v>
-      </c>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="5"/>
+        <v>1.014910062303704</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0.051104129752821</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>11.035197839997357</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>26.75</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>0.749881599168729</v>
+      </c>
       <c r="J22" s="2" t="n">
-        <v>80388</v>
+        <v>8606</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>448</v>
+        <v>902</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>vitamin_c</v>
+        <v>vitamin_d</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>0.750962170993504</v>
+        <v>0.751939056653897</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0.555603704809794</v>
+        <v>0.345901924260547</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>1.014910062303704</v>
+        <v>1.634439610946421</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>0.051104129752821</v>
+        <v>0.038515484547745</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>11.035197839997357</v>
+        <v>14.680130642537975</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>26.75</v>
+        <v>98.12</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>0.749881599168729</v>
+        <v>0.010681367030405</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>8606</v>
+        <v>339695</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>902</v>
+        <v>4466</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>vitamin_d</v>
+        <v>vitamin_e</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>0.751939056653897</v>
+        <v>0.763761279522364</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>0.345901924260547</v>
+        <v>0.583098006241082</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>1.634439610946421</v>
+        <v>1.0003000450045</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>0.038515484547745</v>
+        <v>0.350245514116019</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>14.680130642537975</v>
+        <v>1.665492543337498</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>98.12</v>
+        <v>43.82</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.010681367030405</v>
+        <v>0.665283345187216</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>339695</v>
+        <v>158299</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>4466</v>
+        <v>1839</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>vitamin_e</v>
+        <v>vitamin_b12</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>0.763761279522364</v>
+        <v>0.7708048744499</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0.583098006241082</v>
+        <v>0.611081981756899</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>1.0003000450045</v>
-      </c>
-      <c r="F25" s="3" t="n">
-        <v>0.350245514116019</v>
-      </c>
-      <c r="G25" s="3" t="n">
-        <v>1.665492543337498</v>
-      </c>
-      <c r="H25" s="4" t="n">
-        <v>43.82</v>
-      </c>
-      <c r="I25" s="5" t="n">
-        <v>0.665283345187216</v>
-      </c>
+        <v>0.990044948040641</v>
+      </c>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="5"/>
       <c r="J25" s="2" t="n">
-        <v>158299</v>
+        <v>2589</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>1839</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>vitamin_b12</v>
+        <v>folic_acid</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>0.7708048744499</v>
+        <v>0.773290880810785</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.611081981756899</v>
+        <v>0.60683400087146</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.990044948040641</v>
-      </c>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="5"/>
+        <v>0.985407517519414</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>0.351608041308591</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>1.700697128881358</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>63.72</v>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>0.291332348940905</v>
+      </c>
       <c r="J26" s="2" t="n">
-        <v>2589</v>
+        <v>309245</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>1171</v>
+        <v>2289</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>folic_acid</v>
+        <v>avocado</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>0.773290880810785</v>
+        <v>0.777322466429106</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>0.60683400087146</v>
+        <v>0.595949110875099</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.985407517519414</v>
-      </c>
-      <c r="F27" s="3" t="n">
-        <v>0.351608041308591</v>
-      </c>
-      <c r="G27" s="3" t="n">
-        <v>1.700697128881358</v>
-      </c>
+        <v>1.013794275030678</v>
+      </c>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
       <c r="H27" s="4" t="n">
-        <v>63.72</v>
-      </c>
-      <c r="I27" s="5" t="n">
-        <v>0.291332348940905</v>
-      </c>
+        <v>20.99</v>
+      </c>
+      <c r="I27" s="5"/>
       <c r="J27" s="2" t="n">
-        <v>309245</v>
+        <v>112328</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>2289</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>avocado</v>
+        <v>dairy</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>0.777322466429106</v>
+        <v>0.8285318499048928</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0.595949110875099</v>
+        <v>0.6515507423707737</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>1.013794275030678</v>
-      </c>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
+        <v>1.0536918026427677</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>0.3820831459958125</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>1.7966378090761093</v>
+      </c>
       <c r="H28" s="4" t="n">
-        <v>20.99</v>
-      </c>
-      <c r="I28" s="5"/>
+        <v>78.58</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>0.13803210241351754</v>
+      </c>
       <c r="J28" s="2" t="n">
-        <v>112328</v>
+        <v>799763</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>1165</v>
+        <v>5469</v>
       </c>
     </row>
     <row r="29">
@@ -1731,37 +1731,31 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>processed_meat_intake</v>
+        <v>ultra_processed_food_intake</v>
       </c>
       <c r="B43" s="2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>1.086433159799911</v>
+        <v>1.0695093586575706</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>0.97921896456946</v>
+        <v>0.9109201832456592</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>1.205265651112213</v>
-      </c>
-      <c r="F43" s="3" t="n">
-        <v>0.838562859743763</v>
-      </c>
-      <c r="G43" s="3" t="n">
-        <v>1.407571295339136</v>
-      </c>
+        <v>1.2557085563529022</v>
+      </c>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
       <c r="H43" s="4" t="n">
-        <v>41.47</v>
-      </c>
-      <c r="I43" s="5" t="n">
-        <v>0.083837824241743</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I43" s="5"/>
       <c r="J43" s="2" t="n">
-        <v>938913</v>
+        <v>647537</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>6956</v>
+        <v>1906</v>
       </c>
     </row>
     <row r="44">
@@ -1793,75 +1787,81 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>sugar_sweetened_beverage_intake</v>
+        <v>processed_meat_intake</v>
       </c>
       <c r="B45" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C45" s="3" t="n">
-        <v>1.109722458890099</v>
+        <v>1.098230227423644</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>1.009977038572974</v>
+        <v>0.9861961589479402</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>1.219390011363415</v>
-      </c>
-      <c r="F45" s="3"/>
-      <c r="G45" s="3"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="5"/>
+        <v>1.2231139195550809</v>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>0.8427431092536752</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>1.4311711590203418</v>
+      </c>
+      <c r="H45" s="4" t="n">
+        <v>42.14</v>
+      </c>
+      <c r="I45" s="5" t="n">
+        <v>0.03309532537024148</v>
+      </c>
       <c r="J45" s="2" t="n">
-        <v>73024</v>
+        <v>939835</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>297</v>
+        <v>6986</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>dietary_protein_intake</v>
+        <v>sugar_sweetened_beverage_intake</v>
       </c>
       <c r="B46" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>1.117841954220713</v>
+        <v>1.109722458890099</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>1.012983563938329</v>
+        <v>1.009977038572974</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>1.233678059956743</v>
+        <v>1.219390011363415</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
-      <c r="H46" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="H46" s="4"/>
       <c r="I46" s="5"/>
       <c r="J46" s="2" t="n">
-        <v>585408</v>
+        <v>73024</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>2402</v>
+        <v>297</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>animal_protein_intake</v>
+        <v>dietary_protein_intake</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>1.151654955944369</v>
+        <v>1.117841954220713</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>1.038211997081825</v>
+        <v>1.012983563938329</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>1.277365814492968</v>
+        <v>1.233678059956743</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
@@ -1878,259 +1878,296 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>tomato</v>
+        <v>animal_protein_intake</v>
       </c>
       <c r="B48" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C48" s="3" t="n">
-        <v>1.19945453907786</v>
+        <v>1.151654955944369</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>0.950107996733684</v>
+        <v>1.038211997081825</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>1.518204486493061</v>
+        <v>1.277365814492968</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
-      <c r="H48" s="4"/>
+      <c r="H48" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="I48" s="5"/>
       <c r="J48" s="2" t="n">
-        <v>101683</v>
+        <v>585408</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>774</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>red_meat</v>
+        <v>calcium</v>
       </c>
       <c r="B49" s="2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C49" s="3" t="n">
-        <v>1.32154300883515</v>
+        <v>1.1698786201893066</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>1.111710699877804</v>
+        <v>0.8336013404157353</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>1.570980583701342</v>
+        <v>1.6419753520733475</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>0.781587403506308</v>
+        <v>0.029223708876296984</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>2.234524144537297</v>
+        <v>46.832385025779665</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>77.01</v>
+        <v>61.22</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>0.01127626650555</v>
+        <v>0.09782654651999097</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>1417360</v>
+        <v>493396</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>6876</v>
+        <v>1881</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>calcium</v>
+        <v>tomato</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C50" s="3" t="n">
-        <v>1.763833989140762</v>
+        <v>1.19945453907786</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>1</v>
+        <v>0.950107996733684</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>3.119550071749652</v>
+        <v>1.518204486493061</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
       <c r="H50" s="4"/>
       <c r="I50" s="5"/>
       <c r="J50" s="2" t="n">
-        <v>586</v>
+        <v>101683</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>200</v>
+        <v>774</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>caffeine</v>
+        <v>red_meat</v>
       </c>
       <c r="B51" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C51" s="3" t="n">
-        <v>2.045114195119933</v>
+        <v>1.32154300883515</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>1.149607920243644</v>
+        <v>1.111710699877804</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>3.637955664073244</v>
-      </c>
-      <c r="F51" s="3"/>
-      <c r="G51" s="3"/>
-      <c r="H51" s="4"/>
-      <c r="I51" s="5"/>
+        <v>1.570980583701342</v>
+      </c>
+      <c r="F51" s="3" t="n">
+        <v>0.781587403506308</v>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>2.234524144537297</v>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>77.01</v>
+      </c>
+      <c r="I51" s="5" t="n">
+        <v>0.01127626650555</v>
+      </c>
       <c r="J51" s="2" t="n">
-        <v>104440</v>
+        <v>1417360</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>206</v>
+        <v>6876</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>pickled_vegetables</v>
+        <v>caffeine</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C52" s="3" t="n">
-        <v>3.217136946095633</v>
+        <v>2.045114195119933</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>1.357780842990217</v>
+        <v>1.149607920243644</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>7.482070687809</v>
+        <v>3.637955664073244</v>
       </c>
       <c r="F52" s="3"/>
       <c r="G52" s="3"/>
       <c r="H52" s="4"/>
       <c r="I52" s="5"/>
       <c r="J52" s="2" t="n">
-        <v>260</v>
+        <v>104440</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>130</v>
+        <v>206</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>vegetable_and_seed_oil_intake</v>
+        <v>pickled_vegetables</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C53" s="3" t="n">
-        <v>3.431519625226634</v>
+        <v>3.217136946095633</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>1.684722438489189</v>
+        <v>1.357780842990217</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>6.946365883186642</v>
+        <v>7.482070687809</v>
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
       <c r="H53" s="4"/>
       <c r="I53" s="5"/>
       <c r="J53" s="2" t="n">
-        <v>405</v>
+        <v>260</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>113</v>
+        <v>130</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>eggs</v>
+        <v>vegetable_and_seed_oil_intake</v>
       </c>
       <c r="B54" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C54" s="3" t="n">
-        <v>3.857811292537815</v>
+        <v>3.431519625226634</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>2.646928735129925</v>
+        <v>1.684722438489189</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>5.622632665288498</v>
+        <v>6.946365883186642</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
-      <c r="H54" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="H54" s="4"/>
       <c r="I54" s="5"/>
       <c r="J54" s="2" t="n">
-        <v>1995</v>
+        <v>405</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>355</v>
+        <v>113</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>soy</v>
+        <v>eggs</v>
       </c>
       <c r="B55" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C55" s="3" t="n">
-        <v>4.61</v>
+        <v>3.857811292537815</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>1.57</v>
+        <v>2.646928735129925</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>13.51</v>
+        <v>5.622632665288498</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
-      <c r="H55" s="4"/>
+      <c r="H55" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="I55" s="5"/>
       <c r="J55" s="2" t="n">
-        <v>18244</v>
+        <v>1995</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>61</v>
+        <v>355</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>anti_inflammatory_diet</v>
+        <v>soy</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C56" s="3" t="n">
-        <v>5.609539624201962</v>
+        <v>4.61</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>1.456957290394739</v>
+        <v>1.57</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>20.449495214599413</v>
+        <v>13.51</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
       <c r="H56" s="4"/>
       <c r="I56" s="5"/>
       <c r="J56" s="2" t="n">
+        <v>18244</v>
+      </c>
+      <c r="K56" s="2" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>anti_inflammatory_diet</v>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" s="3" t="n">
+        <v>5.609539624201962</v>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>1.456957290394739</v>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>20.449495214599413</v>
+      </c>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="4"/>
+      <c r="I57" s="5"/>
+      <c r="J57" s="2" t="n">
         <v>199</v>
       </c>
-      <c r="K56" s="2" t="n">
+      <c r="K57" s="2" t="n">
         <v>95</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K56"/>
+  <autoFilter ref="A1:K57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>